<commit_message>
Fix email addresses invented from prose, and record the campaign send
The obfuscated-email reader matched "at" and "dot" inside ordinary words, so
it manufactured addresses for creators who never published one: the bio link
detoxheather.com became detoxhe@her.com ("he-AT-her"), and "health educator.
Ask your doctor" became educ@or.ask. Three of the 141 addresses were fabricated
this way and would have been mailed.

Separators must now be standalone tokens, and a result whose TLD is not one
people actually use in a bio is rejected. Caught before the send; the list is
138 real addresses, 134 of them sendable.

Also records the send: nine BCC blobs, one per competitor anchor plus generic
and Spanish, each threaded to Adam's inbox, with thread ids stored so replies
can be attributed back to a segment.
</commit_message>
<xml_diff>
--- a/data/output/colostrum_creator_list.xlsx
+++ b/data/output/colostrum_creator_list.xlsx
@@ -23630,11 +23630,7 @@
       <c r="C155" t="n">
         <v>76100</v>
       </c>
-      <c r="D155" t="inlineStr">
-        <is>
-          <t>educ@or.ask</t>
-        </is>
-      </c>
+      <c r="D155" t="inlineStr"/>
       <c r="E155" t="inlineStr">
         <is>
           <t>English</t>
@@ -25088,11 +25084,7 @@
       <c r="C176" t="n">
         <v>90300</v>
       </c>
-      <c r="D176" t="inlineStr">
-        <is>
-          <t>detoxhe@her.com</t>
-        </is>
-      </c>
+      <c r="D176" t="inlineStr"/>
       <c r="E176" t="inlineStr">
         <is>
           <t>English</t>
@@ -32192,11 +32184,7 @@
       <c r="C282" t="n">
         <v>8192</v>
       </c>
-      <c r="D282" t="inlineStr">
-        <is>
-          <t>www.scaledcre@or.com</t>
-        </is>
-      </c>
+      <c r="D282" t="inlineStr"/>
       <c r="E282" t="inlineStr">
         <is>
           <t>English</t>
@@ -59136,11 +59124,6 @@
       <c r="C201" t="n">
         <v>76100</v>
       </c>
-      <c r="D201" t="inlineStr">
-        <is>
-          <t>educ@or.ask</t>
-        </is>
-      </c>
       <c r="E201" t="n">
         <v>49</v>
       </c>
@@ -61919,11 +61902,6 @@
       <c r="C233" t="n">
         <v>90300</v>
       </c>
-      <c r="D233" t="inlineStr">
-        <is>
-          <t>detoxhe@her.com</t>
-        </is>
-      </c>
       <c r="E233" t="n">
         <v>29</v>
       </c>
@@ -77606,11 +77584,6 @@
       </c>
       <c r="C413" t="n">
         <v>8192</v>
-      </c>
-      <c r="D413" t="inlineStr">
-        <is>
-          <t>www.scaledcre@or.com</t>
-        </is>
       </c>
       <c r="E413" t="n">
         <v>1</v>

</xml_diff>